<commit_message>
Rename general bivariate feedback category
</commit_message>
<xml_diff>
--- a/data/a305_content_analysis.xlsx
+++ b/data/a305_content_analysis.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A305 content analysis" sheetId="1" r:id="R78f4fbbec4fe4065"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A305 content analysis" sheetId="1" r:id="Rb169432adff94b0b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -146,9 +146,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">(“very easy to pinpoint SNR at specific site”)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">General</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">(“hard to make sense from overall”)</x:t>
@@ -1323,11 +1320,11 @@
       <x:c r="A24" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B24" t="s">
+      <x:c r="B24" t="str">
+        <x:v>General bivariates</x:v>
+      </x:c>
+      <x:c r="C24" t="s">
         <x:v>46</x:v>
-      </x:c>
-      <x:c r="C24" t="s">
-        <x:v>47</x:v>
       </x:c>
       <x:c r="D24" t="s">
         <x:v>12</x:v>
@@ -1344,7 +1341,7 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="C25" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="D25" t="s">
         <x:v>7</x:v>
@@ -1361,7 +1358,7 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="C26" t="s">
-        <x:v>49</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D26" t="s">
         <x:v>18</x:v>
@@ -1374,11 +1371,11 @@
       <x:c r="A27" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="B27" t="s">
-        <x:v>46</x:v>
+      <x:c r="B27" t="str">
+        <x:v>General bivariates</x:v>
       </x:c>
       <x:c r="C27" t="s">
-        <x:v>50</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="D27" t="s">
         <x:v>32</x:v>
@@ -1395,10 +1392,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C28" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="D28" t="s">
         <x:v>51</x:v>
-      </x:c>
-      <x:c r="D28" t="s">
-        <x:v>52</x:v>
       </x:c>
       <x:c r="E28" t="s">
         <x:v>8</x:v>
@@ -1412,7 +1409,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C29" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="D29" t="s">
         <x:v>14</x:v>
@@ -1429,7 +1426,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C30" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="D30" t="s">
         <x:v>12</x:v>
@@ -1446,10 +1443,10 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C31" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="D31" t="s">
         <x:v>55</x:v>
-      </x:c>
-      <x:c r="D31" t="s">
-        <x:v>56</x:v>
       </x:c>
       <x:c r="E31" t="s">
         <x:v>15</x:v>
@@ -1463,7 +1460,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C32" t="s">
-        <x:v>57</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="D32" t="s">
         <x:v>12</x:v>
@@ -1480,10 +1477,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C33" t="s">
-        <x:v>58</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="D33" t="s">
-        <x:v>52</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="E33" t="s">
         <x:v>8</x:v>
@@ -1497,7 +1494,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C34" t="s">
-        <x:v>59</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="D34" t="s">
         <x:v>7</x:v>
@@ -1514,7 +1511,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C35" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="D35" t="s">
         <x:v>12</x:v>
@@ -1531,7 +1528,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C36" t="s">
-        <x:v>61</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="D36" t="s">
         <x:v>7</x:v>
@@ -1548,7 +1545,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C37" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="D37" t="s">
         <x:v>12</x:v>
@@ -1565,7 +1562,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C38" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="D38" t="s">
         <x:v>12</x:v>
@@ -1582,7 +1579,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C39" t="s">
-        <x:v>63</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="D39" t="s">
         <x:v>12</x:v>
@@ -1595,11 +1592,11 @@
       <x:c r="A40" t="n">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B40" t="s">
-        <x:v>46</x:v>
+      <x:c r="B40" t="str">
+        <x:v>General bivariates</x:v>
       </x:c>
       <x:c r="C40" t="s">
-        <x:v>64</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="D40" t="s">
         <x:v>32</x:v>
@@ -1616,7 +1613,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C41" t="s">
-        <x:v>65</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="D41" t="s">
         <x:v>25</x:v>
@@ -1633,7 +1630,7 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="C42" t="s">
-        <x:v>65</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="D42" t="s">
         <x:v>25</x:v>
@@ -1650,7 +1647,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C43" t="s">
-        <x:v>65</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="D43" t="s">
         <x:v>25</x:v>
@@ -1667,7 +1664,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="C44" t="s">
-        <x:v>66</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="D44" t="s">
         <x:v>14</x:v>
@@ -1684,7 +1681,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C45" t="s">
-        <x:v>67</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="D45" t="s">
         <x:v>12</x:v>
@@ -1701,7 +1698,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C46" t="s">
-        <x:v>67</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="D46" t="s">
         <x:v>12</x:v>
@@ -1718,7 +1715,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C47" t="s">
-        <x:v>68</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D47" t="s">
         <x:v>28</x:v>
@@ -1731,11 +1728,11 @@
       <x:c r="A48" t="n">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="B48" t="s">
-        <x:v>46</x:v>
+      <x:c r="B48" t="str">
+        <x:v>General bivariates</x:v>
       </x:c>
       <x:c r="C48" t="s">
-        <x:v>69</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="D48" t="s">
         <x:v>12</x:v>
@@ -1752,7 +1749,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C49" t="s">
-        <x:v>70</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D49" t="s">
         <x:v>12</x:v>
@@ -1769,10 +1766,10 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C50" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="D50" t="s">
-        <x:v>52</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="E50" t="s">
         <x:v>26</x:v>
@@ -1782,11 +1779,11 @@
       <x:c r="A51" t="n">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B51" t="s">
-        <x:v>46</x:v>
+      <x:c r="B51" t="str">
+        <x:v>General bivariates</x:v>
       </x:c>
       <x:c r="C51" t="s">
-        <x:v>72</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="D51" t="s">
         <x:v>18</x:v>
@@ -1803,7 +1800,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C52" t="s">
-        <x:v>73</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="D52" t="s">
         <x:v>32</x:v>
@@ -1820,7 +1817,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C53" t="s">
-        <x:v>74</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="D53" t="s">
         <x:v>12</x:v>
@@ -1833,11 +1830,11 @@
       <x:c r="A54" t="n">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="B54" t="s">
-        <x:v>46</x:v>
+      <x:c r="B54" t="str">
+        <x:v>General bivariates</x:v>
       </x:c>
       <x:c r="C54" t="s">
-        <x:v>75</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="D54" t="s">
         <x:v>12</x:v>
@@ -1854,7 +1851,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C55" t="s">
-        <x:v>76</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="D55" t="s">
         <x:v>10</x:v>
@@ -1871,7 +1868,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="C56" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D56" t="s">
         <x:v>12</x:v>
@@ -1888,7 +1885,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C57" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D57" t="s">
         <x:v>12</x:v>
@@ -1905,7 +1902,7 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="C58" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D58" t="s">
         <x:v>12</x:v>
@@ -1922,10 +1919,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C59" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="D59" t="s">
         <x:v>78</x:v>
-      </x:c>
-      <x:c r="D59" t="s">
-        <x:v>79</x:v>
       </x:c>
       <x:c r="E59" t="s">
         <x:v>8</x:v>
@@ -1939,10 +1936,10 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C60" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="D60" t="s">
         <x:v>78</x:v>
-      </x:c>
-      <x:c r="D60" t="s">
-        <x:v>79</x:v>
       </x:c>
       <x:c r="E60" t="s">
         <x:v>8</x:v>
@@ -1956,7 +1953,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C61" t="s">
-        <x:v>80</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="D61" t="s">
         <x:v>12</x:v>
@@ -1973,7 +1970,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C62" t="s">
-        <x:v>81</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="D62" t="s">
         <x:v>14</x:v>
@@ -1990,7 +1987,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C63" t="s">
-        <x:v>82</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="D63" t="s">
         <x:v>7</x:v>
@@ -2007,7 +2004,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C64" t="s">
-        <x:v>83</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="D64" t="s">
         <x:v>28</x:v>
@@ -2024,7 +2021,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C65" t="s">
-        <x:v>84</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="D65" t="s">
         <x:v>7</x:v>
@@ -2041,7 +2038,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C66" t="s">
-        <x:v>85</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="D66" t="s">
         <x:v>32</x:v>
@@ -2058,7 +2055,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C67" t="s">
-        <x:v>86</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D67" t="s">
         <x:v>28</x:v>
@@ -2075,7 +2072,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C68" t="s">
-        <x:v>87</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="D68" t="s">
         <x:v>25</x:v>
@@ -2092,7 +2089,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C69" t="s">
-        <x:v>88</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="D69" t="s">
         <x:v>32</x:v>
@@ -2109,10 +2106,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="C70" t="s">
-        <x:v>89</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="D70" t="s">
-        <x:v>79</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="E70" t="s">
         <x:v>19</x:v>
@@ -2126,7 +2123,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C71" t="s">
-        <x:v>90</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="D71" t="s">
         <x:v>21</x:v>
@@ -2143,7 +2140,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C72" t="s">
-        <x:v>91</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="D72" t="s">
         <x:v>28</x:v>
@@ -2160,7 +2157,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C73" t="s">
-        <x:v>92</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="D73" t="s">
         <x:v>14</x:v>
@@ -2177,7 +2174,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C74" t="s">
-        <x:v>93</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="D74" t="s">
         <x:v>28</x:v>
@@ -2194,7 +2191,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C75" t="s">
-        <x:v>94</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="D75" t="s">
         <x:v>12</x:v>
@@ -2211,7 +2208,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C76" t="s">
-        <x:v>94</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="D76" t="s">
         <x:v>12</x:v>
@@ -2228,7 +2225,7 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="C77" t="s">
-        <x:v>95</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="D77" t="s">
         <x:v>12</x:v>
@@ -2245,7 +2242,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C78" t="s">
-        <x:v>96</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="D78" t="s">
         <x:v>28</x:v>
@@ -2262,7 +2259,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C79" t="s">
-        <x:v>97</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="D79" t="s">
         <x:v>21</x:v>
@@ -2279,7 +2276,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C80" t="s">
-        <x:v>98</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="D80" t="s">
         <x:v>37</x:v>
@@ -2292,11 +2289,11 @@
       <x:c r="A81" t="n">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="B81" t="s">
-        <x:v>46</x:v>
+      <x:c r="B81" t="str">
+        <x:v>General bivariates</x:v>
       </x:c>
       <x:c r="C81" t="s">
-        <x:v>99</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="D81" t="s">
         <x:v>21</x:v>
@@ -2313,7 +2310,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C82" t="s">
-        <x:v>100</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="D82" t="s">
         <x:v>10</x:v>
@@ -2330,7 +2327,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C83" t="s">
-        <x:v>100</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="D83" t="s">
         <x:v>10</x:v>
@@ -2347,7 +2344,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C84" t="s">
-        <x:v>101</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="D84" t="s">
         <x:v>21</x:v>
@@ -2364,7 +2361,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C85" t="s">
-        <x:v>101</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="D85" t="s">
         <x:v>21</x:v>
@@ -2381,7 +2378,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C86" t="s">
-        <x:v>102</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="D86" t="s">
         <x:v>28</x:v>
@@ -2398,7 +2395,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C87" t="s">
-        <x:v>103</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="D87" t="s">
         <x:v>32</x:v>
@@ -2415,7 +2412,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C88" t="s">
-        <x:v>104</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="D88" t="s">
         <x:v>12</x:v>
@@ -2432,7 +2429,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C89" t="s">
-        <x:v>105</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="D89" t="s">
         <x:v>12</x:v>
@@ -2449,7 +2446,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="C90" t="s">
-        <x:v>106</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="D90" t="s">
         <x:v>14</x:v>
@@ -2466,7 +2463,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C91" t="s">
-        <x:v>107</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="D91" t="s">
         <x:v>12</x:v>
@@ -2483,7 +2480,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C92" t="s">
-        <x:v>108</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="D92" t="s">
         <x:v>32</x:v>
@@ -2500,7 +2497,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C93" t="s">
-        <x:v>109</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="D93" t="s">
         <x:v>12</x:v>
@@ -2517,10 +2514,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C94" t="s">
-        <x:v>110</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="D94" t="s">
-        <x:v>52</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="E94" t="s">
         <x:v>8</x:v>
@@ -2534,10 +2531,10 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C95" t="s">
-        <x:v>111</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="D95" t="s">
-        <x:v>52</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="E95" t="s">
         <x:v>8</x:v>
@@ -2551,7 +2548,7 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="C96" t="s">
-        <x:v>112</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="D96" t="s">
         <x:v>12</x:v>
@@ -2568,7 +2565,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C97" t="s">
-        <x:v>113</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="D97" t="s">
         <x:v>12</x:v>
@@ -2585,10 +2582,10 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C98" t="s">
-        <x:v>114</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="D98" t="s">
-        <x:v>79</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="E98" t="s">
         <x:v>15</x:v>
@@ -2602,7 +2599,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C99" t="s">
-        <x:v>115</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="D99" t="s">
         <x:v>7</x:v>
@@ -2619,7 +2616,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C100" t="s">
-        <x:v>116</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="D100" t="s">
         <x:v>37</x:v>
@@ -2636,7 +2633,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C101" t="s">
-        <x:v>117</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="D101" t="s">
         <x:v>32</x:v>
@@ -2653,7 +2650,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C102" t="s">
-        <x:v>117</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="D102" t="s">
         <x:v>32</x:v>
@@ -2670,10 +2667,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C103" t="s">
-        <x:v>118</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="D103" t="s">
-        <x:v>52</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="E103" t="s">
         <x:v>8</x:v>
@@ -2687,7 +2684,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C104" t="s">
-        <x:v>119</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="D104" t="s">
         <x:v>37</x:v>
@@ -2704,7 +2701,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C105" t="s">
-        <x:v>120</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="D105" t="s">
         <x:v>21</x:v>
@@ -2721,7 +2718,7 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="C106" t="s">
-        <x:v>121</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="D106" t="s">
         <x:v>18</x:v>
@@ -2738,7 +2735,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C107" t="s">
-        <x:v>122</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="D107" t="s">
         <x:v>32</x:v>
@@ -2755,7 +2752,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C108" t="s">
-        <x:v>123</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="D108" t="s">
         <x:v>14</x:v>
@@ -2772,10 +2769,10 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C109" t="s">
-        <x:v>124</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="D109" t="s">
-        <x:v>79</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="E109" t="s">
         <x:v>15</x:v>
@@ -2789,7 +2786,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C110" t="s">
-        <x:v>125</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="D110" t="s">
         <x:v>12</x:v>
@@ -2806,7 +2803,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C111" t="s">
-        <x:v>126</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="D111" t="s">
         <x:v>7</x:v>
@@ -2823,7 +2820,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C112" t="s">
-        <x:v>126</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="D112" t="s">
         <x:v>7</x:v>
@@ -2840,7 +2837,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C113" t="s">
-        <x:v>127</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="D113" t="s">
         <x:v>37</x:v>
@@ -2857,10 +2854,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C114" t="s">
-        <x:v>128</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="D114" t="s">
-        <x:v>52</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="E114" t="s">
         <x:v>15</x:v>
@@ -2874,10 +2871,10 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="C115" t="s">
-        <x:v>128</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="D115" t="s">
-        <x:v>52</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="E115" t="s">
         <x:v>15</x:v>
@@ -2891,7 +2888,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C116" t="s">
-        <x:v>129</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="D116" t="s">
         <x:v>25</x:v>
@@ -2908,7 +2905,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C117" t="s">
-        <x:v>130</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="D117" t="s">
         <x:v>21</x:v>
@@ -2925,7 +2922,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C118" t="s">
-        <x:v>131</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="D118" t="s">
         <x:v>21</x:v>
@@ -2942,7 +2939,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C119" t="s">
-        <x:v>132</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="D119" t="s">
         <x:v>37</x:v>
@@ -2959,7 +2956,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C120" t="s">
-        <x:v>133</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="D120" t="s">
         <x:v>37</x:v>
@@ -2976,7 +2973,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C121" t="s">
-        <x:v>134</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="D121" t="s">
         <x:v>18</x:v>
@@ -2993,7 +2990,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C122" t="s">
-        <x:v>135</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="D122" t="s">
         <x:v>10</x:v>
@@ -3010,7 +3007,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C123" t="s">
-        <x:v>136</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="D123" t="s">
         <x:v>21</x:v>
@@ -3027,7 +3024,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C124" t="s">
-        <x:v>136</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="D124" t="s">
         <x:v>21</x:v>
@@ -3044,7 +3041,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C125" t="s">
-        <x:v>137</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="D125" t="s">
         <x:v>12</x:v>
@@ -3061,7 +3058,7 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="C126" t="s">
-        <x:v>138</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="D126" t="s">
         <x:v>32</x:v>
@@ -3078,7 +3075,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C127" t="s">
-        <x:v>139</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="D127" t="s">
         <x:v>37</x:v>
@@ -3095,7 +3092,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C128" t="s">
-        <x:v>140</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="D128" t="s">
         <x:v>12</x:v>
@@ -3112,7 +3109,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="C129" t="s">
-        <x:v>141</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="D129" t="s">
         <x:v>12</x:v>
@@ -3129,7 +3126,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="C130" t="s">
-        <x:v>142</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="D130" t="s">
         <x:v>25</x:v>
@@ -3146,7 +3143,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C131" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="D131" t="s">
         <x:v>21</x:v>
@@ -3163,7 +3160,7 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="C132" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="D132" t="s">
         <x:v>21</x:v>
@@ -3180,7 +3177,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C133" t="s">
-        <x:v>144</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="D133" t="s">
         <x:v>14</x:v>
@@ -3197,7 +3194,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C134" t="s">
-        <x:v>145</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="D134" t="s">
         <x:v>28</x:v>
@@ -3214,7 +3211,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C135" t="s">
-        <x:v>146</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="D135" t="s">
         <x:v>12</x:v>
@@ -3231,7 +3228,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C136" t="s">
-        <x:v>147</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="D136" t="s">
         <x:v>7</x:v>
@@ -3248,7 +3245,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C137" t="s">
-        <x:v>148</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="D137" t="s">
         <x:v>7</x:v>
@@ -3265,10 +3262,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="C138" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="D138" t="s">
-        <x:v>79</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="E138" t="s">
         <x:v>19</x:v>
@@ -3282,7 +3279,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C139" t="s">
-        <x:v>150</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="D139" t="s">
         <x:v>25</x:v>
@@ -3299,7 +3296,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C140" t="s">
-        <x:v>151</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="D140" t="s">
         <x:v>12</x:v>
@@ -3316,7 +3313,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C141" t="s">
-        <x:v>151</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="D141" t="s">
         <x:v>12</x:v>
@@ -3333,7 +3330,7 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="C142" t="s">
-        <x:v>152</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="D142" t="s">
         <x:v>14</x:v>
@@ -3350,7 +3347,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C143" t="s">
-        <x:v>153</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="D143" t="s">
         <x:v>14</x:v>
@@ -3367,7 +3364,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C144" t="s">
-        <x:v>154</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="D144" t="s">
         <x:v>7</x:v>
@@ -3384,7 +3381,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C145" t="s">
-        <x:v>155</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="D145" t="s">
         <x:v>12</x:v>
@@ -3397,11 +3394,11 @@
       <x:c r="A146" t="n">
         <x:v>67</x:v>
       </x:c>
-      <x:c r="B146" t="s">
-        <x:v>46</x:v>
+      <x:c r="B146" t="str">
+        <x:v>General bivariates</x:v>
       </x:c>
       <x:c r="C146" t="s">
-        <x:v>156</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="D146" t="s">
         <x:v>10</x:v>
@@ -3414,14 +3411,14 @@
       <x:c r="A147" t="n">
         <x:v>67</x:v>
       </x:c>
-      <x:c r="B147" t="s">
-        <x:v>46</x:v>
+      <x:c r="B147" t="str">
+        <x:v>General bivariates</x:v>
       </x:c>
       <x:c r="C147" t="s">
-        <x:v>157</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="D147" t="s">
-        <x:v>79</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="E147" t="s">
         <x:v>19</x:v>
@@ -3435,10 +3432,10 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="C148" t="s">
-        <x:v>158</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="D148" t="s">
-        <x:v>79</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="E148" t="s">
         <x:v>19</x:v>
@@ -3452,10 +3449,10 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C149" t="s">
-        <x:v>159</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="D149" t="s">
-        <x:v>79</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="E149" t="s">
         <x:v>15</x:v>
@@ -3469,10 +3466,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C150" t="s">
-        <x:v>160</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="D150" t="s">
-        <x:v>79</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="E150" t="s">
         <x:v>15</x:v>
@@ -3486,10 +3483,10 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C151" t="s">
-        <x:v>160</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="D151" t="s">
-        <x:v>79</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="E151" t="s">
         <x:v>15</x:v>
@@ -3503,7 +3500,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C152" t="s">
-        <x:v>161</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="D152" t="s">
         <x:v>12</x:v>
@@ -3520,7 +3517,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C153" t="s">
-        <x:v>162</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="D153" t="s">
         <x:v>12</x:v>
@@ -3537,10 +3534,10 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C154" t="s">
-        <x:v>163</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="D154" t="s">
-        <x:v>79</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="E154" t="s">
         <x:v>8</x:v>
@@ -3554,7 +3551,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C155" t="s">
-        <x:v>164</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="D155" t="s">
         <x:v>28</x:v>
@@ -3571,7 +3568,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C156" t="s">
-        <x:v>164</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="D156" t="s">
         <x:v>28</x:v>
@@ -3588,7 +3585,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C157" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="D157" t="s">
         <x:v>10</x:v>
@@ -3605,7 +3602,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C158" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="D158" t="s">
         <x:v>10</x:v>
@@ -3622,7 +3619,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C159" t="s">
-        <x:v>166</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="D159" t="s">
         <x:v>21</x:v>
@@ -3639,7 +3636,7 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="C160" t="s">
-        <x:v>167</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="D160" t="s">
         <x:v>7</x:v>
@@ -3656,7 +3653,7 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="C161" t="s">
-        <x:v>168</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="D161" t="s">
         <x:v>12</x:v>
@@ -3673,7 +3670,7 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="C162" t="s">
-        <x:v>169</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="D162" t="s">
         <x:v>32</x:v>
@@ -3690,7 +3687,7 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="C163" t="s">
-        <x:v>170</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="D163" t="s">
         <x:v>28</x:v>
@@ -3707,7 +3704,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C164" t="s">
-        <x:v>171</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="D164" t="s">
         <x:v>12</x:v>
@@ -3724,7 +3721,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C165" t="s">
-        <x:v>171</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="D165" t="s">
         <x:v>12</x:v>
@@ -3741,7 +3738,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C166" t="s">
-        <x:v>171</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="D166" t="s">
         <x:v>12</x:v>
@@ -3758,7 +3755,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C167" t="s">
-        <x:v>172</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="D167" t="s">
         <x:v>28</x:v>
@@ -3775,13 +3772,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C168" t="s">
-        <x:v>173</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="D168" t="s">
         <x:v>7</x:v>
       </x:c>
       <x:c r="E168" t="s">
-        <x:v>174</x:v>
+        <x:v>173</x:v>
       </x:c>
     </x:row>
     <x:row r="169">
@@ -3792,7 +3789,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="C169" t="s">
-        <x:v>175</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="D169" t="s">
         <x:v>12</x:v>
@@ -3809,7 +3806,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="C170" t="s">
-        <x:v>176</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="D170" t="s">
         <x:v>18</x:v>
@@ -3826,7 +3823,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C171" t="s">
-        <x:v>177</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="D171" t="s">
         <x:v>10</x:v>
@@ -3843,7 +3840,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C172" t="s">
-        <x:v>178</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="D172" t="s">
         <x:v>28</x:v>
@@ -3860,7 +3857,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C173" t="s">
-        <x:v>179</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="D173" t="s">
         <x:v>28</x:v>
@@ -3877,10 +3874,10 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C174" t="s">
-        <x:v>180</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="D174" t="s">
-        <x:v>52</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="E174" t="s">
         <x:v>8</x:v>
@@ -3894,7 +3891,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C175" t="s">
-        <x:v>181</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="D175" t="s">
         <x:v>14</x:v>
@@ -3911,7 +3908,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C176" t="s">
-        <x:v>182</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="D176" t="s">
         <x:v>32</x:v>
@@ -3928,7 +3925,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C177" t="s">
-        <x:v>183</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="D177" t="s">
         <x:v>14</x:v>
@@ -3945,7 +3942,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C178" t="s">
-        <x:v>184</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="D178" t="s">
         <x:v>21</x:v>
@@ -3962,7 +3959,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C179" t="s">
-        <x:v>184</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="D179" t="s">
         <x:v>21</x:v>
@@ -3979,7 +3976,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C180" t="s">
-        <x:v>185</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="D180" t="s">
         <x:v>37</x:v>
@@ -3996,7 +3993,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C181" t="s">
-        <x:v>186</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="D181" t="s">
         <x:v>28</x:v>
@@ -4013,7 +4010,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C182" t="s">
-        <x:v>187</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="D182" t="s">
         <x:v>32</x:v>
@@ -4030,7 +4027,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C183" t="s">
-        <x:v>188</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="D183" t="s">
         <x:v>28</x:v>
@@ -4047,7 +4044,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C184" t="s">
-        <x:v>189</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="D184" t="s">
         <x:v>14</x:v>
@@ -4064,7 +4061,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C185" t="s">
-        <x:v>190</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="D185" t="s">
         <x:v>32</x:v>
@@ -4081,7 +4078,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C186" t="s">
-        <x:v>191</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="D186" t="s">
         <x:v>12</x:v>
@@ -4098,7 +4095,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C187" t="s">
-        <x:v>192</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="D187" t="s">
         <x:v>32</x:v>
@@ -4115,7 +4112,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C188" t="s">
-        <x:v>193</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="D188" t="s">
         <x:v>12</x:v>
@@ -4132,7 +4129,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C189" t="s">
-        <x:v>194</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="D189" t="s">
         <x:v>12</x:v>
@@ -4149,10 +4146,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C190" t="s">
-        <x:v>195</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="D190" t="s">
-        <x:v>56</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="E190" t="s">
         <x:v>15</x:v>
@@ -4166,7 +4163,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C191" t="s">
-        <x:v>196</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="D191" t="s">
         <x:v>28</x:v>
@@ -4183,7 +4180,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C192" t="s">
-        <x:v>197</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="D192" t="s">
         <x:v>12</x:v>
@@ -4200,7 +4197,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C193" t="s">
-        <x:v>198</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="D193" t="s">
         <x:v>7</x:v>
@@ -4213,11 +4210,11 @@
       <x:c r="A194" t="n">
         <x:v>94</x:v>
       </x:c>
-      <x:c r="B194" t="s">
-        <x:v>46</x:v>
+      <x:c r="B194" t="str">
+        <x:v>General bivariates</x:v>
       </x:c>
       <x:c r="C194" t="s">
-        <x:v>199</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="D194" t="s">
         <x:v>10</x:v>
@@ -4234,7 +4231,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C195" t="s">
-        <x:v>200</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="D195" t="s">
         <x:v>7</x:v>
@@ -4251,7 +4248,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C196" t="s">
-        <x:v>201</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="D196" t="s">
         <x:v>37</x:v>
@@ -4268,7 +4265,7 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="C197" t="s">
-        <x:v>202</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="D197" t="s">
         <x:v>12</x:v>
@@ -4285,10 +4282,10 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C198" t="s">
-        <x:v>203</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="D198" t="s">
-        <x:v>79</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="E198" t="s">
         <x:v>26</x:v>
@@ -4302,7 +4299,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C199" t="s">
-        <x:v>204</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="D199" t="s">
         <x:v>18</x:v>
@@ -4319,7 +4316,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C200" t="s">
-        <x:v>205</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="D200" t="s">
         <x:v>28</x:v>
@@ -4336,7 +4333,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C201" t="s">
-        <x:v>206</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="D201" t="s">
         <x:v>37</x:v>
@@ -4353,7 +4350,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C202" t="s">
-        <x:v>207</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="D202" t="s">
         <x:v>10</x:v>
@@ -4370,7 +4367,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C203" t="s">
-        <x:v>208</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="D203" t="s">
         <x:v>12</x:v>
@@ -4387,7 +4384,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="C204" t="s">
-        <x:v>209</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="D204" t="s">
         <x:v>12</x:v>
@@ -4404,7 +4401,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C205" t="s">
-        <x:v>210</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="D205" t="s">
         <x:v>21</x:v>
@@ -4421,7 +4418,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C206" t="s">
-        <x:v>211</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="D206" t="s">
         <x:v>12</x:v>
@@ -4438,7 +4435,7 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="C207" t="s">
-        <x:v>212</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="D207" t="s">
         <x:v>12</x:v>
@@ -4455,7 +4452,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C208" t="s">
-        <x:v>212</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="D208" t="s">
         <x:v>12</x:v>
@@ -4472,7 +4469,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="C209" t="s">
-        <x:v>213</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="D209" t="s">
         <x:v>28</x:v>
@@ -4489,7 +4486,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C210" t="s">
-        <x:v>214</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="D210" t="s">
         <x:v>37</x:v>
@@ -4506,10 +4503,10 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="C211" t="s">
-        <x:v>215</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="D211" t="s">
-        <x:v>79</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="E211" t="s">
         <x:v>19</x:v>
@@ -4523,13 +4520,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C212" t="s">
-        <x:v>216</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="D212" t="s">
-        <x:v>79</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="E212" t="s">
-        <x:v>174</x:v>
+        <x:v>173</x:v>
       </x:c>
     </x:row>
     <x:row r="213">
@@ -4540,7 +4537,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C213" t="s">
-        <x:v>217</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="D213" t="s">
         <x:v>12</x:v>
@@ -4557,7 +4554,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C214" t="s">
-        <x:v>217</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="D214" t="s">
         <x:v>12</x:v>
@@ -4639,7 +4636,7 @@
         <x:v>107</x:v>
       </x:c>
       <x:c r="B219" t="str">
-        <x:v>General</x:v>
+        <x:v>General bivariates</x:v>
       </x:c>
       <x:c r="C219" t="str">
         <x:v>(“the bivariate color plots are still uncommon, but I could get used to them”)</x:v>
@@ -4656,7 +4653,7 @@
         <x:v>107</x:v>
       </x:c>
       <x:c r="B220" t="str">
-        <x:v>General</x:v>
+        <x:v>General bivariates</x:v>
       </x:c>
       <x:c r="C220" t="str">
         <x:v>(“I prefer the more flashy colors”)</x:v>
@@ -4758,7 +4755,7 @@
         <x:v>111</x:v>
       </x:c>
       <x:c r="B226" t="str">
-        <x:v>General</x:v>
+        <x:v>General bivariates</x:v>
       </x:c>
       <x:c r="C226" t="str">
         <x:v>(“voltage and standard error visualisations generally helpful”)</x:v>
@@ -4792,7 +4789,7 @@
         <x:v>111</x:v>
       </x:c>
       <x:c r="B228" t="str">
-        <x:v>General</x:v>
+        <x:v>General bivariates</x:v>
       </x:c>
       <x:c r="C228" t="str">
         <x:v>(“combined two-dimensional colour visualisation useful once I understood the legend”)</x:v>
@@ -4809,7 +4806,7 @@
         <x:v>111</x:v>
       </x:c>
       <x:c r="B229" t="str">
-        <x:v>General</x:v>
+        <x:v>General bivariates</x:v>
       </x:c>
       <x:c r="C229" t="str">
         <x:v>(“presented both pieces of information in a single plot”)</x:v>
@@ -4826,7 +4823,7 @@
         <x:v>111</x:v>
       </x:c>
       <x:c r="B230" t="str">
-        <x:v>General</x:v>
+        <x:v>General bivariates</x:v>
       </x:c>
       <x:c r="C230" t="str">
         <x:v>(“required more attention”)</x:v>
@@ -4843,7 +4840,7 @@
         <x:v>111</x:v>
       </x:c>
       <x:c r="B231" t="str">
-        <x:v>General</x:v>
+        <x:v>General bivariates</x:v>
       </x:c>
       <x:c r="C231" t="str">
         <x:v>(“initially less intuitive than viewing voltage and SE separately”)</x:v>
@@ -4860,7 +4857,7 @@
         <x:v>111</x:v>
       </x:c>
       <x:c r="B232" t="str">
-        <x:v>General</x:v>
+        <x:v>General bivariates</x:v>
       </x:c>
       <x:c r="C232" t="str">
         <x:v>(“clear colour scales and consistent spatial layouts were especially helpful for comparing regions accurately”)</x:v>
@@ -4877,7 +4874,7 @@
         <x:v>112</x:v>
       </x:c>
       <x:c r="B233" t="str">
-        <x:v>General</x:v>
+        <x:v>General bivariates</x:v>
       </x:c>
       <x:c r="C233" t="str">
         <x:v>(“I like the concept of”)</x:v>
@@ -4894,7 +4891,7 @@
         <x:v>112</x:v>
       </x:c>
       <x:c r="B234" t="str">
-        <x:v>General</x:v>
+        <x:v>General bivariates</x:v>
       </x:c>
       <x:c r="C234" t="str">
         <x:v>(“I found them are are to interpret”)</x:v>
@@ -4945,7 +4942,7 @@
         <x:v>112</x:v>
       </x:c>
       <x:c r="B237" t="str">
-        <x:v>General</x:v>
+        <x:v>General bivariates</x:v>
       </x:c>
       <x:c r="C237" t="str">
         <x:v>(“I already find them easier to interpret now that I've finished the tasks”)</x:v>
@@ -5028,7 +5025,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R295fe604bbb640f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6fd2caf73d02416f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>